<commit_message>
Refresh monthly cost workbook
</commit_message>
<xml_diff>
--- a/monthly cost.xlsx
+++ b/monthly cost.xlsx
@@ -463,7 +463,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="4">
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>46112</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="5">

</xml_diff>